<commit_message>
changed the exp_database folder
</commit_message>
<xml_diff>
--- a/exp_database/test_JAQOS/RGB1_Morpho_Manual.xlsx
+++ b/exp_database/test_JAQOS/RGB1_Morpho_Manual.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3801" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3801" uniqueCount="61">
   <si>
     <t xml:space="preserve">Measuring Date</t>
   </si>
@@ -197,6 +197,9 @@
   </si>
   <si>
     <t xml:space="preserve">2024_ToAB_Stress_80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Huachano</t>
   </si>
   <si>
     <t xml:space="preserve">2024_ToAB_Stress_81</t>
@@ -6023,7 +6026,7 @@
         <v>23</v>
       </c>
       <c r="I83" s="4" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="J83" s="5" t="s">
         <v>25</v>
@@ -6088,7 +6091,7 @@
         <v>23</v>
       </c>
       <c r="I84" s="4" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="J84" s="5" t="s">
         <v>25</v>
@@ -6153,7 +6156,7 @@
         <v>23</v>
       </c>
       <c r="I85" s="4" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="J85" s="5" t="s">
         <v>25</v>
@@ -6206,10 +6209,10 @@
         <v>3</v>
       </c>
       <c r="E86" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G86" s="5" t="s">
         <v>22</v>
@@ -6271,10 +6274,10 @@
         <v>3</v>
       </c>
       <c r="E87" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G87" s="19" t="s">
         <v>22</v>
@@ -6336,10 +6339,10 @@
         <v>3</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G88" s="19" t="s">
         <v>22</v>
@@ -6401,10 +6404,10 @@
         <v>3</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G89" s="5" t="s">
         <v>22</v>
@@ -6466,10 +6469,10 @@
         <v>3</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G90" s="19" t="s">
         <v>22</v>
@@ -6531,10 +6534,10 @@
         <v>3</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G91" s="5" t="s">
         <v>22</v>
@@ -9131,10 +9134,10 @@
         <v>4</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G131" s="5" t="s">
         <v>22</v>
@@ -9196,10 +9199,10 @@
         <v>4</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G132" s="5" t="s">
         <v>22</v>
@@ -9261,10 +9264,10 @@
         <v>4</v>
       </c>
       <c r="E133" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G133" s="5" t="s">
         <v>22</v>
@@ -9326,10 +9329,10 @@
         <v>4</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G134" s="5" t="s">
         <v>22</v>
@@ -9391,10 +9394,10 @@
         <v>4</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G135" s="5" t="s">
         <v>22</v>
@@ -9456,10 +9459,10 @@
         <v>4</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G136" s="5" t="s">
         <v>22</v>
@@ -14981,10 +14984,10 @@
         <v>5</v>
       </c>
       <c r="E221" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F221" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G221" s="5" t="s">
         <v>22</v>
@@ -15046,10 +15049,10 @@
         <v>5</v>
       </c>
       <c r="E222" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F222" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G222" s="5" t="s">
         <v>22</v>
@@ -15111,10 +15114,10 @@
         <v>5</v>
       </c>
       <c r="E223" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F223" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G223" s="5" t="s">
         <v>22</v>
@@ -15176,10 +15179,10 @@
         <v>5</v>
       </c>
       <c r="E224" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F224" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G224" s="5" t="s">
         <v>22</v>
@@ -15241,10 +15244,10 @@
         <v>5</v>
       </c>
       <c r="E225" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F225" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G225" s="5" t="s">
         <v>22</v>
@@ -15306,10 +15309,10 @@
         <v>5</v>
       </c>
       <c r="E226" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F226" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G226" s="5" t="s">
         <v>22</v>
@@ -23756,10 +23759,10 @@
         <v>6</v>
       </c>
       <c r="E356" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F356" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G356" s="5" t="s">
         <v>22</v>
@@ -23821,10 +23824,10 @@
         <v>6</v>
       </c>
       <c r="E357" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F357" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G357" s="5" t="s">
         <v>22</v>
@@ -23886,10 +23889,10 @@
         <v>6</v>
       </c>
       <c r="E358" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F358" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G358" s="5" t="s">
         <v>22</v>
@@ -23951,10 +23954,10 @@
         <v>6</v>
       </c>
       <c r="E359" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F359" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G359" s="5" t="s">
         <v>22</v>
@@ -24016,10 +24019,10 @@
         <v>6</v>
       </c>
       <c r="E360" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F360" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G360" s="5" t="s">
         <v>22</v>
@@ -24081,10 +24084,10 @@
         <v>6</v>
       </c>
       <c r="E361" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F361" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G361" s="5" t="s">
         <v>22</v>
@@ -29606,10 +29609,10 @@
         <v>7</v>
       </c>
       <c r="E446" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F446" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G446" s="5" t="s">
         <v>22</v>
@@ -29671,10 +29674,10 @@
         <v>7</v>
       </c>
       <c r="E447" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F447" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G447" s="5" t="s">
         <v>22</v>
@@ -29736,10 +29739,10 @@
         <v>7</v>
       </c>
       <c r="E448" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F448" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G448" s="5" t="s">
         <v>22</v>
@@ -29801,10 +29804,10 @@
         <v>7</v>
       </c>
       <c r="E449" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F449" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G449" s="5" t="s">
         <v>22</v>
@@ -29866,10 +29869,10 @@
         <v>7</v>
       </c>
       <c r="E450" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F450" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G450" s="5" t="s">
         <v>22</v>
@@ -29931,10 +29934,10 @@
         <v>7</v>
       </c>
       <c r="E451" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F451" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G451" s="5" t="s">
         <v>22</v>

</xml_diff>